<commit_message>
Apply forensic audit fixes to compliance and workbook files
</commit_message>
<xml_diff>
--- a/customer-delivery/06 - Pricing and Calculators/07 - Business Pricing Calculators.xlsx
+++ b/customer-delivery/06 - Pricing and Calculators/07 - Business Pricing Calculators.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="$0.00"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -123,8 +123,23 @@
       <color rgb="000F2547"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000000FF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00666666"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -154,6 +169,11 @@
         <fgColor rgb="00FAF8F4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -189,7 +209,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -332,6 +352,14 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="16" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -428,6 +456,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -909,11 +940,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="22" min="1" max="1"/>
     <col width="15" customWidth="1" style="22" min="2" max="7"/>
+    <col width="22" customWidth="1" style="23" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" s="23">
@@ -929,6 +961,16 @@
           <t>Blue text = enter your own numbers here. Black text = calculates automatically. Do not edit black cells.</t>
         </is>
       </c>
+      <c r="H2" s="49" t="inlineStr">
+        <is>
+          <t>Employer burden assumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="H3" s="50" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="4" ht="26.25" customHeight="1" s="23">
       <c r="A4" s="33" t="inlineStr">
@@ -958,7 +1000,7 @@
       </c>
       <c r="F4" s="33" t="inlineStr">
         <is>
-          <t>Monthly burden (18%)</t>
+          <t>Monthly employer burden</t>
         </is>
       </c>
       <c r="G4" s="33" t="inlineStr">
@@ -988,7 +1030,7 @@
         <v/>
       </c>
       <c r="F5" s="35">
-        <f>E5*0.18</f>
+        <f>E5*$H$3</f>
         <v/>
       </c>
       <c r="G5" s="35">
@@ -1017,7 +1059,7 @@
         <v/>
       </c>
       <c r="F6" s="35">
-        <f>E6*0.18</f>
+        <f>E6*$H$3</f>
         <v/>
       </c>
       <c r="G6" s="35">
@@ -1046,7 +1088,7 @@
         <v/>
       </c>
       <c r="F7" s="35">
-        <f>E7*0.18</f>
+        <f>E7*$H$3</f>
         <v/>
       </c>
       <c r="G7" s="35">
@@ -1075,7 +1117,7 @@
         <v/>
       </c>
       <c r="F8" s="35">
-        <f>E8*0.18</f>
+        <f>E8*$H$3</f>
         <v/>
       </c>
       <c r="G8" s="35">
@@ -1104,7 +1146,7 @@
         <v/>
       </c>
       <c r="F9" s="35">
-        <f>E9*0.18</f>
+        <f>E9*$H$3</f>
         <v/>
       </c>
       <c r="G9" s="35">
@@ -1133,7 +1175,7 @@
         <v/>
       </c>
       <c r="F10" s="35">
-        <f>E10*0.18</f>
+        <f>E10*$H$3</f>
         <v/>
       </c>
       <c r="G10" s="35">
@@ -1190,6 +1232,18 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="51" t="inlineStr">
+        <is>
+          <t>Employer burden rate</t>
+        </is>
+      </c>
+      <c r="B15" s="52" t="inlineStr">
+        <is>
+          <t>Enter your own combined employer-cost assumption (payroll taxes, workers' compensation, and other employer burden as applicable). Default is 15% for illustration; verify with your payroll provider/accountant.</t>
+        </is>
+      </c>
+    </row>
     <row r="16" ht="32" customHeight="1" s="23">
       <c r="A16" s="41" t="inlineStr">
         <is>
@@ -1198,11 +1252,12 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="B15:G16"/>
     <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A14:C14"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>